<commit_message>
Format and Update ProductBacklog_group51.xlsx
</commit_message>
<xml_diff>
--- a/documents/ProductBacklog_group51.xlsx
+++ b/documents/ProductBacklog_group51.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g726\Desktop\叮咚鸡\Recruitment-System-for-TA\documents\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C2E339-7A6B-4E47-8975-011FAB439974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="163">
   <si>
     <t>Story ID</t>
   </si>
@@ -285,8 +291,8 @@
 So that I can maintain system security and integrity.</t>
   </si>
   <si>
-    <t>1. Admin can view list of users
-2. Admin can deactivate or delete user accounts
+    <t>1. Admin can view list of users_x000D_
+2. Admin can deactivate or delete user accounts_x000D_
 3. Admin can view user roles</t>
   </si>
   <si>
@@ -301,8 +307,8 @@
 So that inappropriate or outdated jobs can be removed.</t>
   </si>
   <si>
-    <t>1. Admin can view all job postings
-2. Admin can edit job information
+    <t>1. Admin can view all job postings_x000D_
+2. Admin can edit job information_x000D_
 3. Admin can delete job postings</t>
   </si>
   <si>
@@ -320,8 +326,8 @@
     <t>Could</t>
   </si>
   <si>
-    <t>1. Admin can export applicant data
-2. Admin can export job application records
+    <t>1. Admin can export applicant data_x000D_
+2. Admin can export job application records_x000D_
 3. Data can be exported as CSV or Excel file</t>
   </si>
   <si>
@@ -541,11 +547,6 @@
     <t>CV Parsing</t>
   </si>
   <si>
-    <t>As a TA applicant
-I want the system to extract skills from my uploaded CV
-So that my applicant profile can be automatically populated.</t>
-  </si>
-  <si>
     <t>1. System analyses uploaded CV text
 2. Skills and education are extracted
 3. Extracted information is stored in applicant profile and can be edited by the user</t>
@@ -560,20 +561,7 @@
     <t>AI applicant ranking</t>
   </si>
   <si>
-    <t>As a module organiser
-I want the system to rank applicants automatically
-So that I can quickly identify the most suitable candidates.</t>
-  </si>
-  <si>
-    <t>1. System analyses CV and job requirements
-2. Applicants receive a ranking score
-3. MO can view ranked applicant list</t>
-  </si>
-  <si>
     <t>AI ranking</t>
-  </si>
-  <si>
-    <t>US-30</t>
   </si>
   <si>
     <t>View Applicant List</t>
@@ -592,18 +580,65 @@
 MO can filter applicants by criteria like skills or status.
 MO can click on an applicant's name to view the full profile.</t>
   </si>
+  <si>
+    <t>US-30</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>US-31</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a module organiser
+I want the system to rank applicants automatically
+So that I can quickly identify the most suitable candidates.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant
+I want the system to extract skills from my uploaded CV
+So that my applicant profile can be automatically populated.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Applications Manage</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant
+I want to view a list of positions I have applied for and adjust their priority order
+So that I can inform the MO which positions I prefer to be assigned to first.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Should</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. System analyses CV and job requirements
+2. Applicants receive a ranking score
+3. MO can view ranked applicant list</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. View List: User can view a list of all submitted TA applications
+2. Status Display: Each entry must show the position name and current status
+3. Reorder: User can change the preference order of applications</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Essential for the algorithm to resolve multiple offers</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="179" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -615,155 +650,17 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <sz val="9"/>
       <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -772,192 +669,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -980,254 +697,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1238,68 +713,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="常规 2" xfId="49"/>
+    <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1497,27 +941,27 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J51"/>
-  <sheetFormatPr defaultColWidth="8.08333333333333" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="8.0625" defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.41666666666667" customWidth="1"/>
+    <col min="1" max="1" width="8.4375" customWidth="1"/>
     <col min="2" max="2" width="15.25" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="40.1666666666667" customWidth="1"/>
-    <col min="7" max="7" width="18.1666666666667" customWidth="1"/>
+    <col min="6" max="6" width="40.1875" customWidth="1"/>
+    <col min="7" max="7" width="18.1875" customWidth="1"/>
     <col min="8" max="8" width="15.75" customWidth="1"/>
     <col min="9" max="9" width="22.75" customWidth="1"/>
-    <col min="10" max="10" width="24.1666666666667" customWidth="1"/>
+    <col min="10" max="10" width="24.1875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48.75" customHeight="1" spans="1:10">
+    <row r="1" spans="1:10" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1549,86 +993,89 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A3" t="s">
+    <row r="3" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I3" t="s">
+      <c r="H3" s="3"/>
+      <c r="I3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A4" t="s">
+    <row r="4" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E4" s="3">
         <v>2</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>2</v>
       </c>
+      <c r="H4" s="3"/>
       <c r="I4" s="4">
         <v>46109</v>
       </c>
@@ -1636,28 +1083,29 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="5" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A5" t="s">
+    <row r="5" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
         <v>2</v>
       </c>
+      <c r="H5" s="3"/>
       <c r="I5" s="4">
         <v>46101</v>
       </c>
@@ -1665,118 +1113,121 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="6" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A6" t="s">
+    <row r="6" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="3">
         <v>2</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="7" t="s">
         <v>35</v>
       </c>
       <c r="G6" s="3">
         <v>4</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A7" t="s">
+    <row r="7" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I7" t="s">
+      <c r="H7" s="3"/>
+      <c r="I7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="J7" s="4">
         <v>46108</v>
       </c>
     </row>
-    <row r="8" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A8" t="s">
+    <row r="8" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I8" t="s">
+      <c r="H8" s="3"/>
+      <c r="I8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A9" t="s">
+    <row r="9" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="3" t="s">
         <v>43</v>
       </c>
+      <c r="H9" s="3"/>
       <c r="I9" s="4">
         <v>46101</v>
       </c>
@@ -1784,762 +1235,800 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="10" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A10" t="s">
+    <row r="10" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="3">
         <v>1</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I10" t="s">
+      <c r="H10" s="3"/>
+      <c r="I10" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A11" t="s">
+    <row r="11" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I11" t="s">
+      <c r="H11" s="3"/>
+      <c r="I11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A12" s="5" t="s">
+    <row r="12" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I12" t="s">
+      <c r="H12" s="3"/>
+      <c r="I12" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I13" t="s">
+      <c r="H13" s="3"/>
+      <c r="I13" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I14" t="s">
+      <c r="H14" s="3"/>
+      <c r="I14" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="9" t="s">
         <v>77</v>
       </c>
       <c r="G15" s="3">
         <v>4</v>
       </c>
-      <c r="I15" t="s">
+      <c r="H15" s="3"/>
+      <c r="I15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A16" s="5" t="s">
+    <row r="16" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="9" t="s">
         <v>81</v>
       </c>
       <c r="G16" s="3">
         <v>3</v>
       </c>
-      <c r="I16" t="s">
+      <c r="H16" s="3"/>
+      <c r="I16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="9" t="s">
         <v>85</v>
       </c>
       <c r="G17" s="3">
         <v>5</v>
       </c>
-      <c r="I17" t="s">
+      <c r="H17" s="3"/>
+      <c r="I17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="18" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="9" t="s">
         <v>91</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I18" t="s">
+      <c r="H18" s="3"/>
+      <c r="I18" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="19" ht="33.5" customHeight="1" spans="1:10">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E19" s="3">
         <v>1</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="9" t="s">
         <v>96</v>
       </c>
       <c r="G19" s="3">
         <v>3</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E20" s="3">
         <v>1</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="7" t="s">
         <v>101</v>
       </c>
       <c r="G20" s="3">
         <v>3</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E21" s="3">
         <v>1</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="7" t="s">
         <v>106</v>
       </c>
       <c r="G21" s="3">
         <v>2</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E22" s="3">
         <v>1</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="9" t="s">
         <v>111</v>
       </c>
       <c r="G22" s="3">
         <v>3</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H22" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="I22" t="s">
+      <c r="I22" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E23" s="3">
         <v>1</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F23" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G23" s="3">
         <v>3</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A24" s="5" t="s">
+    <row r="24" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E24" s="3">
         <v>2</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="7" t="s">
         <v>121</v>
       </c>
       <c r="G24" s="3">
         <v>2</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A25" s="5" t="s">
+    <row r="25" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E25" s="3">
         <v>2</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="7" t="s">
         <v>126</v>
       </c>
       <c r="G25" s="3">
         <v>3</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H25" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I25" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="26" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A26" s="5" t="s">
+    <row r="26" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E26" s="3">
         <v>2</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="7" t="s">
         <v>131</v>
       </c>
       <c r="G26" s="3">
         <v>3</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H26" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I26" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="27" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E27" s="3">
         <v>2</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" s="7" t="s">
         <v>136</v>
       </c>
       <c r="G27" s="3">
         <v>2</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="28" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A28" s="5" t="s">
+    <row r="28" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="3" t="s">
         <v>76</v>
       </c>
       <c r="E28" s="3">
         <v>3</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F28" s="9" t="s">
         <v>141</v>
       </c>
       <c r="G28" s="3">
         <v>5</v>
       </c>
-      <c r="H28" s="5" t="s">
+      <c r="H28" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="I28" t="s">
+      <c r="I28" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J28" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="29" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="C29" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>76</v>
       </c>
       <c r="E29" s="3">
         <v>3</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>146</v>
+      <c r="F29" s="9" t="s">
+        <v>145</v>
       </c>
       <c r="G29" s="3">
         <v>5</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H29" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="I29" t="s">
-        <v>86</v>
-      </c>
-      <c r="J29" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="30" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A30" s="5" t="s">
+      <c r="B30" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B30" t="s">
-        <v>149</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="C30" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>76</v>
       </c>
       <c r="E30" s="3">
         <v>3</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>151</v>
+      <c r="F30" s="9" t="s">
+        <v>160</v>
       </c>
       <c r="G30" s="3">
         <v>5</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="H30" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" s="3">
+        <v>1</v>
+      </c>
+      <c r="F31" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="I30" t="s">
-        <v>86</v>
-      </c>
-      <c r="J30" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="31" ht="34.15" customHeight="1" spans="1:10">
-      <c r="A31" t="s">
-        <v>153</v>
-      </c>
-      <c r="B31" t="s">
-        <v>154</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D31" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31">
-        <v>1</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="G31">
+      <c r="G31" s="3">
         <v>5</v>
       </c>
-      <c r="I31" s="4">
+      <c r="H31" s="3"/>
+      <c r="I31" s="5">
         <v>46101</v>
       </c>
       <c r="J31" s="4">
         <v>46108</v>
       </c>
     </row>
-    <row r="32" ht="34.15" customHeight="1" spans="1:10">
-      <c r="C32" s="2"/>
-      <c r="F32" s="2"/>
-    </row>
-    <row r="33" ht="34.15" customHeight="1" spans="3:6">
+    <row r="32" spans="1:10" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="E32" s="3">
+        <v>3</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="G32" s="3">
+        <v>3</v>
+      </c>
+      <c r="H32" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="I32" s="4">
+        <v>46118</v>
+      </c>
+      <c r="J32" s="6">
+        <v>46127</v>
+      </c>
+    </row>
+    <row r="33" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C33" s="2"/>
       <c r="F33" s="2"/>
     </row>
-    <row r="34" ht="34.15" customHeight="1" spans="3:6">
+    <row r="34" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C34" s="2"/>
       <c r="F34" s="2"/>
     </row>
-    <row r="35" ht="34.15" customHeight="1" spans="3:6">
+    <row r="35" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C35" s="2"/>
       <c r="F35" s="2"/>
     </row>
-    <row r="36" ht="34.15" customHeight="1" spans="3:6">
+    <row r="36" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C36" s="2"/>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" ht="34.15" customHeight="1" spans="3:6">
+    <row r="37" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C37" s="2"/>
       <c r="F37" s="2"/>
     </row>
-    <row r="38" ht="34.15" customHeight="1" spans="3:6">
+    <row r="38" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C38" s="2"/>
       <c r="F38" s="2"/>
     </row>
-    <row r="39" ht="34.15" customHeight="1" spans="3:6">
+    <row r="39" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C39" s="2"/>
       <c r="F39" s="2"/>
     </row>
-    <row r="40" ht="34.15" customHeight="1" spans="3:6">
+    <row r="40" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C40" s="2"/>
       <c r="F40" s="2"/>
     </row>
-    <row r="41" ht="34.15" customHeight="1" spans="3:6">
+    <row r="41" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C41" s="2"/>
       <c r="F41" s="2"/>
     </row>
-    <row r="42" ht="34.15" customHeight="1" spans="3:6">
+    <row r="42" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C42" s="2"/>
       <c r="F42" s="2"/>
     </row>
-    <row r="43" ht="34.15" customHeight="1" spans="3:6">
+    <row r="43" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C43" s="2"/>
       <c r="F43" s="2"/>
     </row>
-    <row r="44" ht="34.15" customHeight="1" spans="3:6">
+    <row r="44" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C44" s="2"/>
       <c r="F44" s="2"/>
     </row>
-    <row r="45" ht="34.15" customHeight="1" spans="3:6">
+    <row r="45" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C45" s="2"/>
       <c r="F45" s="2"/>
     </row>
-    <row r="46" ht="34.15" customHeight="1" spans="3:6">
+    <row r="46" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C46" s="2"/>
       <c r="F46" s="2"/>
     </row>
-    <row r="47" ht="34.15" customHeight="1" spans="3:6">
+    <row r="47" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C47" s="2"/>
       <c r="F47" s="2"/>
     </row>
-    <row r="48" ht="34.15" customHeight="1" spans="3:6">
+    <row r="48" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C48" s="2"/>
       <c r="F48" s="2"/>
     </row>
-    <row r="49" ht="34.15" customHeight="1" spans="3:6">
+    <row r="49" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C49" s="2"/>
       <c r="F49" s="2"/>
     </row>
-    <row r="50" ht="34.15" customHeight="1" spans="3:6">
+    <row r="50" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C50" s="2"/>
       <c r="F50" s="2"/>
     </row>
-    <row r="51" ht="34.15" customHeight="1" spans="3:6">
+    <row r="51" spans="3:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F51" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>